<commit_message>
Updated Row validation and user Validation in Attendance File
</commit_message>
<xml_diff>
--- a/test.xlsx
+++ b/test.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aagam\Documents\Gituhub\FYP-material\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6465CFC-2158-4037-87D6-0932BECC1F37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B1B5BC8-B964-4127-AF70-FB634F97EB52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="12">
   <si>
     <t>Name</t>
   </si>
@@ -47,21 +47,12 @@
     <t>Date</t>
   </si>
   <si>
-    <t>Grade 1</t>
-  </si>
-  <si>
     <t>Absent</t>
   </si>
   <si>
     <t>Present</t>
   </si>
   <si>
-    <t>Aagaman Mainali</t>
-  </si>
-  <si>
-    <t>aagamanmainali35@gmail.com</t>
-  </si>
-  <si>
     <t>Anmol</t>
   </si>
   <si>
@@ -77,7 +68,7 @@
     <t>Grade 10</t>
   </si>
   <si>
-    <t>kjh Status</t>
+    <t>Attendance Status</t>
   </si>
 </sst>
 </file>
@@ -480,305 +471,63 @@
         <v>3</v>
       </c>
       <c r="E1" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>8</v>
       </c>
       <c r="C2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D2" s="1">
+        <f t="shared" ref="D2:D3" ca="1" si="0">TODAY()</f>
+        <v>45761</v>
+      </c>
+      <c r="E2" t="s">
         <v>4</v>
-      </c>
-      <c r="D2" s="1">
-        <v>45750</v>
-      </c>
-      <c r="E2" t="s">
-        <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B3" s="3" t="s">
-        <v>11</v>
-      </c>
       <c r="C3" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="D3" s="1">
-        <v>45750</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>45761</v>
       </c>
       <c r="E3" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>10</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="C4" t="s">
-        <v>13</v>
-      </c>
-      <c r="D4" s="1">
-        <v>45750</v>
-      </c>
-      <c r="E4" t="s">
-        <v>6</v>
-      </c>
+      <c r="D4"/>
     </row>
-    <row r="5" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>10</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="C5" t="s">
-        <v>13</v>
-      </c>
-      <c r="D5" s="1">
-        <f ca="1">TODAY()</f>
-        <v>45760</v>
-      </c>
-      <c r="E5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>7</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="C6" t="s">
-        <v>13</v>
-      </c>
-      <c r="D6" s="1">
-        <f t="shared" ref="D6:D7" ca="1" si="0">TODAY()</f>
-        <v>45760</v>
-      </c>
-      <c r="E6" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>9</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C7" t="s">
-        <v>13</v>
-      </c>
-      <c r="D7" s="1">
-        <f t="shared" ca="1" si="0"/>
-        <v>45760</v>
-      </c>
-      <c r="E7" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>10</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="C8" t="s">
-        <v>13</v>
-      </c>
-      <c r="D8" s="1">
-        <v>45753</v>
-      </c>
-      <c r="E8" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>7</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="C9" t="s">
-        <v>13</v>
-      </c>
-      <c r="D9" s="1">
-        <v>45753</v>
-      </c>
-      <c r="E9" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>9</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C10" t="s">
-        <v>13</v>
-      </c>
-      <c r="D10" s="1">
-        <v>45753</v>
-      </c>
-      <c r="E10" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>10</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="C11" t="s">
-        <v>13</v>
-      </c>
-      <c r="D11" s="1">
-        <v>45754</v>
-      </c>
-      <c r="E11" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
-        <v>7</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="C12" t="s">
-        <v>13</v>
-      </c>
-      <c r="D12" s="1">
-        <v>45754</v>
-      </c>
-      <c r="E12" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
-        <v>9</v>
-      </c>
-      <c r="B13" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C13" t="s">
-        <v>13</v>
-      </c>
-      <c r="D13" s="1">
-        <v>45754</v>
-      </c>
-      <c r="E13" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
-        <v>7</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="C14" t="s">
-        <v>13</v>
-      </c>
-      <c r="D14" s="1">
-        <v>45757</v>
-      </c>
-      <c r="E14" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
-        <v>7</v>
-      </c>
-      <c r="B15" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="C15" t="s">
-        <v>13</v>
-      </c>
-      <c r="D15" s="1">
-        <v>45760</v>
-      </c>
-      <c r="E15" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A16" t="s">
-        <v>9</v>
-      </c>
-      <c r="B16" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C16" t="s">
-        <v>13</v>
-      </c>
-      <c r="D16" s="1">
-        <v>45760</v>
-      </c>
-      <c r="E16" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" t="s">
-        <v>10</v>
-      </c>
-      <c r="B17" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="C17" t="s">
-        <v>13</v>
-      </c>
-      <c r="D17" s="1">
-        <v>45760</v>
-      </c>
-      <c r="E17" t="s">
-        <v>6</v>
-      </c>
-    </row>
+    <row r="5" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="6" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="7" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="8" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="9" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="10" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="11" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
   <hyperlinks>
-    <hyperlink ref="B2" r:id="rId1" xr:uid="{CDD0A97C-5541-45D8-B250-394AE43F38DC}"/>
-    <hyperlink ref="B3" r:id="rId2" xr:uid="{64AD9803-E100-4C8B-B611-54C89DCE8334}"/>
-    <hyperlink ref="B4" r:id="rId3" xr:uid="{49BF50F0-0195-4B89-A9BD-9096E5F527FD}"/>
-    <hyperlink ref="B5" r:id="rId4" xr:uid="{C6A0257E-6123-4E7D-8039-FA2CBA2A2EC4}"/>
-    <hyperlink ref="B6" r:id="rId5" xr:uid="{99AB868C-8B66-406E-9C9B-9A8A253C4C93}"/>
-    <hyperlink ref="B7" r:id="rId6" xr:uid="{6F9F9EFE-8D40-4EA3-9002-3760A91AB1B5}"/>
-    <hyperlink ref="B8" r:id="rId7" xr:uid="{401511D1-2C34-4B4B-9B55-404C37225FD3}"/>
-    <hyperlink ref="B9" r:id="rId8" xr:uid="{194E0D2A-2374-4BC5-9B8A-25A4F12BFF71}"/>
-    <hyperlink ref="B10" r:id="rId9" xr:uid="{391F05C4-2F8E-4EEA-843E-C5B9363B12C6}"/>
-    <hyperlink ref="B11" r:id="rId10" xr:uid="{E6FBF1BB-D226-4241-931E-2175EE706466}"/>
-    <hyperlink ref="B12" r:id="rId11" xr:uid="{D63467FF-2FB4-4138-9513-2D7927DB0316}"/>
-    <hyperlink ref="B13" r:id="rId12" xr:uid="{D9E6BDB6-35E3-46F7-8C28-A1F42B0370F1}"/>
-    <hyperlink ref="B14" r:id="rId13" xr:uid="{BE6885B5-A397-4FF0-BEB0-C49E2802D03E}"/>
-    <hyperlink ref="B15" r:id="rId14" xr:uid="{94710826-0908-4C42-8E66-D30739098AE1}"/>
-    <hyperlink ref="B16" r:id="rId15" xr:uid="{DEACC63A-B278-42E8-B1D6-8F5018C3D75D}"/>
-    <hyperlink ref="B17" r:id="rId16" xr:uid="{1FC2B35B-4B2F-4E5B-BEB7-98E7E5E0CAD2}"/>
+    <hyperlink ref="B2" r:id="rId1" xr:uid="{64AD9803-E100-4C8B-B611-54C89DCE8334}"/>
+    <hyperlink ref="B3" r:id="rId2" xr:uid="{49BF50F0-0195-4B89-A9BD-9096E5F527FD}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId17"/>
+  <pageSetup orientation="portrait" r:id="rId3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Completed all the backedn for FYP
</commit_message>
<xml_diff>
--- a/test.xlsx
+++ b/test.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aagam\Documents\Gituhub\FYP-material\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B1B5BC8-B964-4127-AF70-FB634F97EB52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12445A10-F2F7-4391-AD05-25A67382E725}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
   <si>
     <t>Name</t>
   </si>
@@ -50,25 +50,16 @@
     <t>Absent</t>
   </si>
   <si>
-    <t>Present</t>
-  </si>
-  <si>
-    <t>Anmol</t>
-  </si>
-  <si>
-    <t>Saman</t>
-  </si>
-  <si>
-    <t>9610ileana@ptct.net</t>
-  </si>
-  <si>
-    <t>tealadina@ptct.net</t>
-  </si>
-  <si>
     <t>Grade 10</t>
   </si>
   <si>
     <t>Attendance Status</t>
+  </si>
+  <si>
+    <t>momoskar</t>
+  </si>
+  <si>
+    <t>aagamanmainali35123@gmail.com</t>
   </si>
 </sst>
 </file>
@@ -471,44 +462,30 @@
         <v>3</v>
       </c>
       <c r="E1" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>8</v>
       </c>
       <c r="C2" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="D2" s="1">
-        <f t="shared" ref="D2:D3" ca="1" si="0">TODAY()</f>
-        <v>45761</v>
+        <f t="shared" ref="D2" ca="1" si="0">TODAY()</f>
+        <v>45774</v>
       </c>
       <c r="E2" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>7</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="C3" t="s">
-        <v>10</v>
-      </c>
-      <c r="D3" s="1">
-        <f t="shared" ca="1" si="0"/>
-        <v>45761</v>
-      </c>
-      <c r="E3" t="s">
-        <v>5</v>
-      </c>
+      <c r="B3" s="3"/>
+      <c r="D3" s="1"/>
     </row>
     <row r="4" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D4"/>
@@ -525,9 +502,8 @@
   <phoneticPr fontId="3" type="noConversion"/>
   <hyperlinks>
     <hyperlink ref="B2" r:id="rId1" xr:uid="{64AD9803-E100-4C8B-B611-54C89DCE8334}"/>
-    <hyperlink ref="B3" r:id="rId2" xr:uid="{49BF50F0-0195-4B89-A9BD-9096E5F527FD}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId3"/>
+  <pageSetup orientation="portrait" r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>